<commit_message>
revamp ui to add inbound/outbound station option; prepare for simulation
</commit_message>
<xml_diff>
--- a/frontend/files/example.xlsx
+++ b/frontend/files/example.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kongy\Desktop\mosaic\files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kongy\Desktop\mosaic\frontend\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32DBB13E-A634-470A-B096-07EAFF2255D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB387FA8-4972-43D5-8365-C56418E8E4D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -30,19 +30,19 @@
     <t>B</t>
   </si>
   <si>
-    <t>P1</t>
-  </si>
-  <si>
-    <t>P2D</t>
-  </si>
-  <si>
-    <t>P2P</t>
-  </si>
-  <si>
     <t>C</t>
   </si>
   <si>
     <t>Obs</t>
+  </si>
+  <si>
+    <t>P1I</t>
+  </si>
+  <si>
+    <t>P2DO</t>
+  </si>
+  <si>
+    <t>P2PO</t>
   </si>
 </sst>
 </file>
@@ -737,13 +737,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E2" s="2">
         <v>16</v>
@@ -787,13 +787,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E3" s="2">
         <v>16</v>
@@ -1046,13 +1046,13 @@
         <v>16</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H8" s="2">
         <v>16</v>
@@ -1096,13 +1096,13 @@
         <v>16</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H9" s="2">
         <v>16</v>
@@ -1146,13 +1146,13 @@
         <v>16</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H10" s="2">
         <v>16</v>
@@ -1196,13 +1196,13 @@
         <v>16</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H11" s="2">
         <v>16</v>
@@ -1600,7 +1600,7 @@
         <v>0</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>0</v>
@@ -1609,7 +1609,7 @@
         <v>0</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G21" s="4" t="s">
         <v>0</v>
@@ -1618,7 +1618,7 @@
         <v>0</v>
       </c>
       <c r="I21" s="5" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J21" s="4" t="s">
         <v>0</v>

</xml_diff>